<commit_message>
Animação e fonte tela; Descrição do produto; Redirecionamento de pagamento via WhatsApp.
</commit_message>
<xml_diff>
--- a/backend/produtos_loja.xlsx
+++ b/backend/produtos_loja.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
+  <fileSharing readOnlyRecommended="1"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09D4DC13-7A6E-4D56-9DCA-3B2B85B29A9E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{041A95C2-42EE-4DD4-ADFD-C5950B7E256D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="14810" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -382,27 +383,18 @@
     <t>assets/img/tres-acafrao.jpeg</t>
   </si>
   <si>
-    <t>assets/img/kit-camomila.jpeg</t>
-  </si>
-  <si>
     <t>assets/img/vela-premium.jpeg</t>
   </si>
   <si>
     <t>assets/img/vela-atacado.jpeg</t>
   </si>
   <si>
-    <t>assets/img/aroma-casa.jpeg</t>
-  </si>
-  <si>
     <t>assets/img/bucha-escalda.jpeg</t>
   </si>
   <si>
     <t>assets/img/bucha-sabonete.jpeg</t>
   </si>
   <si>
-    <t>assets/img/vela-sabonete.jpeg</t>
-  </si>
-  <si>
     <t>assets/img/vela-camomila.jpeg</t>
   </si>
   <si>
@@ -410,6 +402,15 @@
   </si>
   <si>
     <t>assets/img/beijavel.jpeg</t>
+  </si>
+  <si>
+    <t>assets/img/aromaecasa.jpeg</t>
+  </si>
+  <si>
+    <t>assets/img/kit-camomila.png</t>
+  </si>
+  <si>
+    <t>assets/img/vela-luxo-luxo.png</t>
   </si>
 </sst>
 </file>
@@ -1035,7 +1036,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="11" spans="1:10" s="3" customFormat="1" ht="50" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" s="3" customFormat="1" ht="37.5" x14ac:dyDescent="0.3">
       <c r="A11" s="10">
         <v>10</v>
       </c>
@@ -1196,7 +1197,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="18" spans="1:7" s="3" customFormat="1" ht="37.5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" s="3" customFormat="1" ht="25" x14ac:dyDescent="0.3">
       <c r="A18" s="10">
         <v>17</v>
       </c>
@@ -1331,7 +1332,7 @@
         <v>54</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
     </row>
     <row r="24" spans="1:7" s="3" customFormat="1" ht="34" customHeight="1" x14ac:dyDescent="0.3">
@@ -1354,7 +1355,7 @@
         <v>52</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="25" spans="1:7" s="3" customFormat="1" ht="37.5" x14ac:dyDescent="0.3">
@@ -1377,7 +1378,7 @@
         <v>52</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="26" spans="1:7" s="3" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -1400,7 +1401,7 @@
         <v>55</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="27" spans="1:7" s="3" customFormat="1" ht="25" x14ac:dyDescent="0.3">
@@ -1423,7 +1424,7 @@
         <v>53</v>
       </c>
       <c r="G27" s="10" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="28" spans="1:7" s="3" customFormat="1" ht="43" customHeight="1" x14ac:dyDescent="0.3">
@@ -1446,7 +1447,7 @@
         <v>52</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="29" spans="1:7" s="3" customFormat="1" ht="37.5" x14ac:dyDescent="0.3">
@@ -1469,10 +1470,10 @@
         <v>52</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" s="3" customFormat="1" ht="50" x14ac:dyDescent="0.3">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" s="3" customFormat="1" ht="37.5" x14ac:dyDescent="0.3">
       <c r="A30" s="10">
         <v>30</v>
       </c>
@@ -1492,7 +1493,7 @@
         <v>52</v>
       </c>
       <c r="G30" s="10" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="31" spans="1:7" s="3" customFormat="1" ht="46" customHeight="1" x14ac:dyDescent="0.3">
@@ -1515,7 +1516,7 @@
         <v>54</v>
       </c>
       <c r="G31" s="10" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="32" spans="1:7" s="3" customFormat="1" ht="25" x14ac:dyDescent="0.3">
@@ -1538,7 +1539,7 @@
         <v>52</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="33" spans="2:6" s="3" customFormat="1" x14ac:dyDescent="0.3">
@@ -1577,5 +1578,8 @@
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="D26:D27 D11" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>